<commit_message>
feat: add DPO regions and nomenclature gender categories
</commit_message>
<xml_diff>
--- a/server/src/modules/startup-import/startup-import.template.xlsx
+++ b/server/src/modules/startup-import/startup-import.template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="82">
   <si>
     <t>Стартовый импорт данных — шаблон</t>
   </si>
@@ -123,6 +123,9 @@
     <t>ФИО руководителя</t>
   </si>
   <si>
+    <t>Регион</t>
+  </si>
+  <si>
     <t>Артикул</t>
   </si>
   <si>
@@ -144,6 +147,9 @@
     <t>Описание</t>
   </si>
   <si>
+    <t>Категория по полу</t>
+  </si>
+  <si>
     <t>ФИО</t>
   </si>
   <si>
@@ -216,6 +222,9 @@
     <t>Новая</t>
   </si>
   <si>
+    <t>Мужское</t>
+  </si>
+  <si>
     <t>Женский</t>
   </si>
   <si>
@@ -228,16 +237,25 @@
     <t>Хорошая</t>
   </si>
   <si>
+    <t>Женское</t>
+  </si>
+  <si>
     <t>headwear</t>
   </si>
   <si>
     <t>Изношенная</t>
   </si>
   <si>
+    <t>Унисекс</t>
+  </si>
+  <si>
     <t>belt</t>
   </si>
   <si>
     <t>Повреждённая</t>
+  </si>
+  <si>
+    <t>Не определено</t>
   </si>
   <si>
     <t>gloves</t>
@@ -864,7 +882,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:H31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -876,7 +894,7 @@
     <col min="7" max="7" width="32" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>28</v>
       </c>
@@ -897,6 +915,9 @@
       </c>
       <c r="G1" s="11" t="s">
         <v>34</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1176,7 +1197,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
@@ -1189,30 +1210,33 @@
     <col min="8" max="8" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
         <v>28</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G1" s="11" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="H1" s="16" t="s">
-        <v>41</v>
+        <v>42</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1563,46 +1587,46 @@
   <sheetData>
     <row r="1" ht="32" customHeight="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="N1" s="11" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -2100,7 +2124,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -2111,27 +2135,27 @@
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="32" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F1" s="11" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="12"/>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -2139,7 +2163,7 @@
       <c r="E2" s="12"/>
       <c r="F2" s="12"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="13"/>
       <c r="B3" s="13"/>
       <c r="C3" s="13"/>
@@ -2147,7 +2171,7 @@
       <c r="E3" s="13"/>
       <c r="F3" s="13"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="13"/>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -2155,7 +2179,7 @@
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="13"/>
       <c r="B5" s="13"/>
       <c r="C5" s="13"/>
@@ -2163,7 +2187,7 @@
       <c r="E5" s="13"/>
       <c r="F5" s="13"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="13"/>
       <c r="B6" s="13"/>
       <c r="C6" s="13"/>
@@ -2171,7 +2195,7 @@
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
       <c r="B7" s="13"/>
       <c r="C7" s="13"/>
@@ -2179,7 +2203,7 @@
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -2187,7 +2211,7 @@
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="13"/>
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
@@ -2195,7 +2219,7 @@
       <c r="E9" s="13"/>
       <c r="F9" s="13"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="13"/>
       <c r="B10" s="13"/>
       <c r="C10" s="13"/>
@@ -2203,7 +2227,7 @@
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="13"/>
       <c r="B11" s="13"/>
       <c r="C11" s="13"/>
@@ -2211,7 +2235,7 @@
       <c r="E11" s="13"/>
       <c r="F11" s="13"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="13"/>
       <c r="B12" s="13"/>
       <c r="C12" s="13"/>
@@ -2219,7 +2243,7 @@
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="13"/>
       <c r="B13" s="13"/>
       <c r="C13" s="13"/>
@@ -2227,7 +2251,7 @@
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="13"/>
       <c r="B14" s="13"/>
       <c r="C14" s="13"/>
@@ -2235,7 +2259,7 @@
       <c r="E14" s="13"/>
       <c r="F14" s="13"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="13"/>
       <c r="B15" s="13"/>
       <c r="C15" s="13"/>
@@ -2243,7 +2267,7 @@
       <c r="E15" s="13"/>
       <c r="F15" s="13"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="13"/>
       <c r="B16" s="13"/>
       <c r="C16" s="13"/>
@@ -2251,7 +2275,7 @@
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="13"/>
       <c r="B17" s="13"/>
       <c r="C17" s="13"/>
@@ -2259,7 +2283,7 @@
       <c r="E17" s="13"/>
       <c r="F17" s="13"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="13"/>
       <c r="B18" s="13"/>
       <c r="C18" s="13"/>
@@ -2267,7 +2291,7 @@
       <c r="E18" s="13"/>
       <c r="F18" s="13"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="13"/>
       <c r="B19" s="13"/>
       <c r="C19" s="13"/>
@@ -2275,7 +2299,7 @@
       <c r="E19" s="13"/>
       <c r="F19" s="13"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="13"/>
       <c r="B20" s="13"/>
       <c r="C20" s="13"/>
@@ -2283,7 +2307,7 @@
       <c r="E20" s="13"/>
       <c r="F20" s="13"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="13"/>
       <c r="B21" s="13"/>
       <c r="C21" s="13"/>
@@ -2291,7 +2315,7 @@
       <c r="E21" s="13"/>
       <c r="F21" s="13"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="13"/>
       <c r="B22" s="13"/>
       <c r="C22" s="13"/>
@@ -2299,7 +2323,7 @@
       <c r="E22" s="13"/>
       <c r="F22" s="13"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23" s="13"/>
       <c r="B23" s="13"/>
       <c r="C23" s="13"/>
@@ -2307,7 +2331,7 @@
       <c r="E23" s="13"/>
       <c r="F23" s="13"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24" s="13"/>
       <c r="B24" s="13"/>
       <c r="C24" s="13"/>
@@ -2315,7 +2339,7 @@
       <c r="E24" s="13"/>
       <c r="F24" s="13"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="13"/>
       <c r="B25" s="13"/>
       <c r="C25" s="13"/>
@@ -2323,7 +2347,7 @@
       <c r="E25" s="13"/>
       <c r="F25" s="13"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="13"/>
       <c r="B26" s="13"/>
       <c r="C26" s="13"/>
@@ -2331,7 +2355,7 @@
       <c r="E26" s="13"/>
       <c r="F26" s="13"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="13"/>
       <c r="B27" s="13"/>
       <c r="C27" s="13"/>
@@ -2339,7 +2363,7 @@
       <c r="E27" s="13"/>
       <c r="F27" s="13"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="13"/>
       <c r="B28" s="13"/>
       <c r="C28" s="13"/>
@@ -2347,7 +2371,7 @@
       <c r="E28" s="13"/>
       <c r="F28" s="13"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="13"/>
       <c r="B29" s="13"/>
       <c r="C29" s="13"/>
@@ -2355,7 +2379,7 @@
       <c r="E29" s="13"/>
       <c r="F29" s="13"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="13"/>
       <c r="B30" s="13"/>
       <c r="C30" s="13"/>
@@ -2363,7 +2387,7 @@
       <c r="E30" s="13"/>
       <c r="F30" s="13"/>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="14"/>
       <c r="B31" s="14"/>
       <c r="C31" s="14"/>
@@ -2406,86 +2430,104 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0"/>
   <cols>
-    <col min="1" max="4" width="28" customWidth="1"/>
+    <col min="1" max="5" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C4" s="20" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D4" s="20" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+      <c r="E4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="21" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B5" s="21" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C5" s="21" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D5" s="21" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+      <c r="E5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="21"/>
       <c r="B6" s="21" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C6" s="21"/>
       <c r="D6" s="21" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+      <c r="E6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="21"/>
       <c r="B7" s="21" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="C7" s="21"/>
       <c r="D7" s="21" t="s">
-        <v>73</v>
+        <v>78</v>
+      </c>
+      <c r="E7" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="21"/>
       <c r="B8" s="21" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C8" s="21"/>
       <c r="D8" s="21"/>
@@ -2493,7 +2535,7 @@
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="21"/>
       <c r="B9" s="21" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C9" s="21"/>
       <c r="D9" s="21"/>

</xml_diff>